<commit_message>
(v2.0.1) fix status and delete netProfit
</commit_message>
<xml_diff>
--- a/frontend/Zakah-calc/public/templates/balance_sheet_template.xlsx
+++ b/frontend/Zakah-calc/public/templates/balance_sheet_template.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java Acadmy\Academy Project\git\Zakah_Project\frontend\Zakah-calc\public\templetes\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF9996F-35C1-420E-A05D-9CC79582B3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DA7D68EF-F2F7-45B9-BAFB-42CC90874FB8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Cash Equivalents</t>
   </si>
@@ -63,9 +57,6 @@
   </si>
   <si>
     <t>Yearly Long Term Liabilities</t>
-  </si>
-  <si>
-    <t>Net Profit</t>
   </si>
   <si>
     <t>Generating Fixed Assets</t>
@@ -80,8 +71,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,7 +163,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -224,7 +215,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -438,31 +429,31 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A57CE91-45F4-459C-8105-5B627B480FFE}">
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.69921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="20.296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.69921875" customWidth="1"/>
+    <col min="12" max="12" width="22.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -496,11 +487,8 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>0</v>
       </c>
@@ -532,9 +520,6 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
         <v>0</v>
       </c>
     </row>

</xml_diff>